<commit_message>
📚 docs: Atualiza README.md
</commit_message>
<xml_diff>
--- a/Tabelas.xlsx
+++ b/Tabelas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\layon\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\layon\Downloads\Problema-de-Localizacao-com-Cobertura-Parcial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB506BE5-A157-49F2-A997-559C6764DB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67F24DC9-21E5-4EE5-A698-89D1B7FCDA71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{792840E6-1BCE-4F5B-B3B2-7B844065BC26}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="2" xr2:uid="{792840E6-1BCE-4F5B-B3B2-7B844065BC26}"/>
   </bookViews>
   <sheets>
     <sheet name="Pequenas" sheetId="1" r:id="rId1"/>
@@ -119,7 +119,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -259,12 +259,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -272,6 +309,90 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -281,92 +402,44 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -692,405 +765,409 @@
     <col min="10" max="10" width="9.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="B1" s="36" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="38"/>
+      <c r="F1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="4" t="s">
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="38"/>
+      <c r="J1" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="39" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2" t="s">
+      <c r="A2" s="42"/>
+      <c r="B2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="5"/>
-      <c r="K2" s="4"/>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="4"/>
+      <c r="A3" s="35"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="41"/>
+      <c r="K3" s="41"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="4">
         <v>73</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="4">
         <v>73</v>
       </c>
-      <c r="D4" s="20">
-        <v>0</v>
-      </c>
-      <c r="E4" s="8">
+      <c r="D4" s="16">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>0.31601977348327642</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="4">
         <v>73</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="4">
         <v>73</v>
       </c>
-      <c r="H4" s="20">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8">
+      <c r="H4" s="16">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5">
         <v>0.20987701416015619</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="4">
         <v>5.5</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="6">
         <v>0.5</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="1">
         <v>68</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="1">
         <v>68</v>
       </c>
-      <c r="D5" s="22">
-        <v>0</v>
-      </c>
-      <c r="E5" s="11">
+      <c r="D5" s="18">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7">
         <v>0.46992754936218262</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="1">
         <v>68</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="1">
         <v>68</v>
       </c>
-      <c r="H5" s="22">
-        <v>0</v>
-      </c>
-      <c r="I5" s="11">
+      <c r="H5" s="18">
+        <v>0</v>
+      </c>
+      <c r="I5" s="7">
         <v>0.39223384857177729</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="1">
         <v>5.75</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="1">
         <v>62</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="1">
         <v>62</v>
       </c>
-      <c r="D6" s="22">
-        <v>0</v>
-      </c>
-      <c r="E6" s="11">
+      <c r="D6" s="18">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7">
         <v>0.194378137588501</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="1">
         <v>62</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="1">
         <v>62</v>
       </c>
-      <c r="H6" s="22">
-        <v>0</v>
-      </c>
-      <c r="I6" s="11">
+      <c r="H6" s="18">
+        <v>0</v>
+      </c>
+      <c r="I6" s="7">
         <v>0.2963566780090332</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="1">
         <v>6</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="1">
         <v>58</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="1">
         <v>58</v>
       </c>
-      <c r="D7" s="22">
-        <v>0</v>
-      </c>
-      <c r="E7" s="11">
+      <c r="D7" s="18">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7">
         <v>0.57574796676635742</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="1">
         <v>58</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="1">
         <v>58</v>
       </c>
-      <c r="H7" s="22">
-        <v>0</v>
-      </c>
-      <c r="I7" s="11">
+      <c r="H7" s="18">
+        <v>0</v>
+      </c>
+      <c r="I7" s="7">
         <v>0.53014373779296875</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="1">
         <v>6.25</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="1">
         <v>69</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="1">
         <v>69</v>
       </c>
-      <c r="D8" s="22">
-        <v>0</v>
-      </c>
-      <c r="E8" s="11">
+      <c r="D8" s="18">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7">
         <v>0.46718740463256841</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="1">
         <v>69</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G8" s="1">
         <v>69</v>
       </c>
-      <c r="H8" s="22">
-        <v>0</v>
-      </c>
-      <c r="I8" s="11">
+      <c r="H8" s="18">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7">
         <v>0.33062505722045898</v>
       </c>
-      <c r="J8" s="10">
+      <c r="J8" s="1">
         <v>5.5</v>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="1">
         <v>64</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="1">
         <v>64</v>
       </c>
-      <c r="D9" s="22">
-        <v>0</v>
-      </c>
-      <c r="E9" s="11">
+      <c r="D9" s="18">
+        <v>0</v>
+      </c>
+      <c r="E9" s="7">
         <v>0.33504676818847662</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="1">
         <v>64</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="1">
         <v>64</v>
       </c>
-      <c r="H9" s="22">
-        <v>0</v>
-      </c>
-      <c r="I9" s="11">
+      <c r="H9" s="18">
+        <v>0</v>
+      </c>
+      <c r="I9" s="7">
         <v>0.70955252647399902</v>
       </c>
-      <c r="J9" s="10">
+      <c r="J9" s="1">
         <v>5.75</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="1">
         <v>61</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="1">
         <v>61</v>
       </c>
-      <c r="D10" s="22">
-        <v>0</v>
-      </c>
-      <c r="E10" s="11">
+      <c r="D10" s="18">
+        <v>0</v>
+      </c>
+      <c r="E10" s="7">
         <v>1.6455023288726811</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="1">
         <v>61</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="1">
         <v>61</v>
       </c>
-      <c r="H10" s="22">
-        <v>0</v>
-      </c>
-      <c r="I10" s="11">
+      <c r="H10" s="18">
+        <v>0</v>
+      </c>
+      <c r="I10" s="7">
         <v>1.2470536231994629</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="1">
         <v>6</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="18" t="s">
+      <c r="A11" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="9">
         <v>50</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="9">
         <v>50</v>
       </c>
-      <c r="D11" s="24">
-        <v>0</v>
-      </c>
-      <c r="E11" s="14">
+      <c r="D11" s="20">
+        <v>0</v>
+      </c>
+      <c r="E11" s="10">
         <v>0.29062962532043463</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="9">
         <v>50</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="9">
         <v>50</v>
       </c>
-      <c r="H11" s="24">
-        <v>0</v>
-      </c>
-      <c r="I11" s="14">
+      <c r="H11" s="20">
+        <v>0</v>
+      </c>
+      <c r="I11" s="10">
         <v>0.20496177673339841</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="9">
         <v>6.25</v>
       </c>
-      <c r="K11" s="15">
+      <c r="K11" s="11">
         <v>0.5</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="27">
-        <f>AVERAGE(B4:B11)</f>
+      <c r="B12" s="23">
+        <f t="shared" ref="B12:I12" si="0">AVERAGE(B4:B11)</f>
         <v>63.125</v>
       </c>
-      <c r="C12" s="27">
-        <f>AVERAGE(C4:C11)</f>
+      <c r="C12" s="23">
+        <f t="shared" si="0"/>
         <v>63.125</v>
       </c>
-      <c r="D12" s="28">
-        <f>AVERAGE(D4:D11)</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="27">
-        <f>AVERAGE(E4:E11)</f>
+      <c r="D12" s="24">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E12" s="23">
+        <f t="shared" si="0"/>
         <v>0.53680494427680969</v>
       </c>
-      <c r="F12" s="27">
-        <f>AVERAGE(F4:F11)</f>
+      <c r="F12" s="23">
+        <f t="shared" si="0"/>
         <v>63.125</v>
       </c>
-      <c r="G12" s="27">
-        <f>AVERAGE(G4:G11)</f>
+      <c r="G12" s="23">
+        <f t="shared" si="0"/>
         <v>63.125</v>
       </c>
-      <c r="H12" s="28">
-        <f>AVERAGE(H4:H11)</f>
-        <v>0</v>
-      </c>
-      <c r="I12" s="27">
-        <f>AVERAGE(I4:I11)</f>
+      <c r="H12" s="24">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I12" s="23">
+        <f t="shared" si="0"/>
         <v>0.49010053277015686</v>
       </c>
+      <c r="J12" s="43"/>
+      <c r="K12" s="44"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J1:J3"/>
     <mergeCell ref="K1:K3"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="F1:I1"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="G2:G3"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1106,391 +1183,392 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="B1" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="4" t="s">
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="32" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2" t="s">
+      <c r="A2" s="31"/>
+      <c r="B2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="5"/>
-      <c r="K2" s="4"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="32"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="4"/>
+      <c r="A3" s="31"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="32"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="4">
         <v>90</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="4">
         <v>90</v>
       </c>
-      <c r="D4" s="20">
-        <v>0</v>
-      </c>
-      <c r="E4" s="8">
+      <c r="D4" s="16">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>2.4942598342895508</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="4">
         <v>90</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="4">
         <v>90</v>
       </c>
-      <c r="H4" s="20">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8">
+      <c r="H4" s="16">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5">
         <v>2.195796012878418</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="4">
         <v>5.5</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="6">
         <v>0.5</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="1">
         <v>79</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="1">
         <v>79</v>
       </c>
-      <c r="D5" s="22">
-        <v>0</v>
-      </c>
-      <c r="E5" s="11">
+      <c r="D5" s="18">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7">
         <v>1.3389656543731689</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="1">
         <v>79</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="1">
         <v>79</v>
       </c>
-      <c r="H5" s="22">
-        <v>0</v>
-      </c>
-      <c r="I5" s="11">
+      <c r="H5" s="18">
+        <v>0</v>
+      </c>
+      <c r="I5" s="7">
         <v>0.84847688674926758</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="1">
         <v>5.75</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="1">
         <v>76</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="1">
         <v>76</v>
       </c>
-      <c r="D6" s="22">
-        <v>0</v>
-      </c>
-      <c r="E6" s="11">
+      <c r="D6" s="18">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7">
         <v>4.7770867347717294</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="1">
         <v>76</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="1">
         <v>76</v>
       </c>
-      <c r="H6" s="22">
-        <v>0</v>
-      </c>
-      <c r="I6" s="11">
+      <c r="H6" s="18">
+        <v>0</v>
+      </c>
+      <c r="I6" s="7">
         <v>4.3617203235626221</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="1">
         <v>6</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="1">
         <v>65</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="1">
         <v>65</v>
       </c>
-      <c r="D7" s="22">
-        <v>0</v>
-      </c>
-      <c r="E7" s="11">
+      <c r="D7" s="18">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7">
         <v>0.93832635879516602</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="1">
         <v>65</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="1">
         <v>65</v>
       </c>
-      <c r="H7" s="22">
-        <v>0</v>
-      </c>
-      <c r="I7" s="11">
+      <c r="H7" s="18">
+        <v>0</v>
+      </c>
+      <c r="I7" s="7">
         <v>0.33417081832885742</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="1">
         <v>6.25</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="1">
         <v>84</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="1">
         <v>84</v>
       </c>
-      <c r="D8" s="22">
-        <v>0</v>
-      </c>
-      <c r="E8" s="11">
+      <c r="D8" s="18">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7">
         <v>2.9015204906463619</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="1">
         <v>84</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G8" s="1">
         <v>84</v>
       </c>
-      <c r="H8" s="22">
-        <v>0</v>
-      </c>
-      <c r="I8" s="11">
+      <c r="H8" s="18">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7">
         <v>1.7795026302337651</v>
       </c>
-      <c r="J8" s="10">
+      <c r="J8" s="1">
         <v>5.5</v>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
+      <c r="A9" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="1">
         <v>75</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="1">
         <v>75</v>
       </c>
-      <c r="D9" s="22">
-        <v>0</v>
-      </c>
-      <c r="E9" s="11">
+      <c r="D9" s="18">
+        <v>0</v>
+      </c>
+      <c r="E9" s="7">
         <v>2.9386458396911621</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="1">
         <v>75</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="1">
         <v>75</v>
       </c>
-      <c r="H9" s="22">
-        <v>0</v>
-      </c>
-      <c r="I9" s="11">
+      <c r="H9" s="18">
+        <v>0</v>
+      </c>
+      <c r="I9" s="7">
         <v>2.9546859264373779</v>
       </c>
-      <c r="J9" s="10">
+      <c r="J9" s="1">
         <v>5.75</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="1">
         <v>65</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="1">
         <v>65</v>
       </c>
-      <c r="D10" s="22">
-        <v>0</v>
-      </c>
-      <c r="E10" s="11">
+      <c r="D10" s="18">
+        <v>0</v>
+      </c>
+      <c r="E10" s="7">
         <v>3.410742044448853</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="1">
         <v>65</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="1">
         <v>65</v>
       </c>
-      <c r="H10" s="22">
-        <v>0</v>
-      </c>
-      <c r="I10" s="11">
+      <c r="H10" s="18">
+        <v>0</v>
+      </c>
+      <c r="I10" s="7">
         <v>4.7275490760803223</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="1">
         <v>6</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="23" t="s">
+      <c r="A11" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="9">
         <v>59</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="9">
         <v>59</v>
       </c>
-      <c r="D11" s="24">
-        <v>0</v>
-      </c>
-      <c r="E11" s="14">
+      <c r="D11" s="20">
+        <v>0</v>
+      </c>
+      <c r="E11" s="10">
         <v>3.616523265838623</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="9">
         <v>59</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="9">
         <v>59</v>
       </c>
-      <c r="H11" s="24">
-        <v>0</v>
-      </c>
-      <c r="I11" s="14">
+      <c r="H11" s="20">
+        <v>0</v>
+      </c>
+      <c r="I11" s="10">
         <v>2.5675351619720459</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="9">
         <v>6.25</v>
       </c>
-      <c r="K11" s="15">
+      <c r="K11" s="11">
         <v>0.5</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="25">
-        <f>AVERAGE(B4:B11)</f>
+      <c r="B12" s="21">
+        <f t="shared" ref="B12:I12" si="0">AVERAGE(B4:B11)</f>
         <v>74.125</v>
       </c>
-      <c r="C12" s="25">
-        <f>AVERAGE(C4:C11)</f>
+      <c r="C12" s="21">
+        <f t="shared" si="0"/>
         <v>74.125</v>
       </c>
-      <c r="D12" s="26">
-        <f>AVERAGE(D4:D11)</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="25">
-        <f>AVERAGE(E4:E11)</f>
+      <c r="D12" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E12" s="21">
+        <f t="shared" si="0"/>
         <v>2.8020087778568268</v>
       </c>
-      <c r="F12" s="25">
-        <f>AVERAGE(F4:F11)</f>
+      <c r="F12" s="21">
+        <f t="shared" si="0"/>
         <v>74.125</v>
       </c>
-      <c r="G12" s="25">
-        <f>AVERAGE(G4:G11)</f>
+      <c r="G12" s="21">
+        <f t="shared" si="0"/>
         <v>74.125</v>
       </c>
-      <c r="H12" s="26">
-        <f>AVERAGE(H4:H11)</f>
-        <v>0</v>
-      </c>
-      <c r="I12" s="25">
-        <f>AVERAGE(I4:I11)</f>
+      <c r="H12" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I12" s="21">
+        <f t="shared" si="0"/>
         <v>2.4711796045303345</v>
       </c>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
+      <c r="J12" s="45"/>
+      <c r="K12" s="46"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
+    <mergeCell ref="J12:K12"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J1:J3"/>
     <mergeCell ref="K1:K3"/>
@@ -1521,397 +1599,392 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2" t="s">
+      <c r="B1" s="31" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="4" t="s">
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="32" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2" t="s">
+      <c r="A2" s="31"/>
+      <c r="B2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="5"/>
-      <c r="K2" s="4"/>
+      <c r="J2" s="33"/>
+      <c r="K2" s="32"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="4"/>
+      <c r="A3" s="31"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="33"/>
+      <c r="K3" s="32"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="4">
         <v>74</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="4">
         <v>74</v>
       </c>
-      <c r="D4" s="20">
-        <v>0</v>
-      </c>
-      <c r="E4" s="8">
+      <c r="D4" s="16">
+        <v>0</v>
+      </c>
+      <c r="E4" s="5">
         <v>13.31495332717896</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="4">
         <v>74</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="4">
         <v>74</v>
       </c>
-      <c r="H4" s="20">
-        <v>0</v>
-      </c>
-      <c r="I4" s="8">
+      <c r="H4" s="16">
+        <v>0</v>
+      </c>
+      <c r="I4" s="5">
         <v>15.40377402305603</v>
       </c>
-      <c r="J4" s="7">
+      <c r="J4" s="4">
         <v>5.5</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="6">
         <v>0.5</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="10">
+      <c r="B5" s="1">
         <v>63</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="1">
         <v>63</v>
       </c>
-      <c r="D5" s="22">
-        <v>0</v>
-      </c>
-      <c r="E5" s="11">
+      <c r="D5" s="18">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7">
         <v>6.0594816207885742</v>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="1">
         <v>63</v>
       </c>
-      <c r="G5" s="10">
+      <c r="G5" s="1">
         <v>63</v>
       </c>
-      <c r="H5" s="22">
-        <v>0</v>
-      </c>
-      <c r="I5" s="11">
+      <c r="H5" s="18">
+        <v>0</v>
+      </c>
+      <c r="I5" s="7">
         <v>4.3675711154937744</v>
       </c>
-      <c r="J5" s="10">
+      <c r="J5" s="1">
         <v>5.75</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="10">
+      <c r="B6" s="1">
         <v>60</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="1">
         <v>60</v>
       </c>
-      <c r="D6" s="22">
-        <v>0</v>
-      </c>
-      <c r="E6" s="11">
+      <c r="D6" s="18">
+        <v>0</v>
+      </c>
+      <c r="E6" s="7">
         <v>12.568864345550541</v>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="1">
         <v>60</v>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="1">
         <v>60</v>
       </c>
-      <c r="H6" s="22">
-        <v>0</v>
-      </c>
-      <c r="I6" s="11">
+      <c r="H6" s="18">
+        <v>0</v>
+      </c>
+      <c r="I6" s="7">
         <v>22.590364456176761</v>
       </c>
-      <c r="J6" s="10">
+      <c r="J6" s="1">
         <v>6</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="33" t="s">
+      <c r="A7" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="10">
+      <c r="B7" s="1">
         <v>48</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="1">
         <v>48</v>
       </c>
-      <c r="D7" s="22">
-        <v>0</v>
-      </c>
-      <c r="E7" s="11">
+      <c r="D7" s="18">
+        <v>0</v>
+      </c>
+      <c r="E7" s="7">
         <v>1.6996510028839109</v>
       </c>
-      <c r="F7" s="10">
+      <c r="F7" s="1">
         <v>48</v>
       </c>
-      <c r="G7" s="10">
+      <c r="G7" s="1">
         <v>48</v>
       </c>
-      <c r="H7" s="22">
-        <v>0</v>
-      </c>
-      <c r="I7" s="11">
+      <c r="H7" s="18">
+        <v>0</v>
+      </c>
+      <c r="I7" s="7">
         <v>1.1308774948120119</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="1">
         <v>6.25</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="1">
         <v>102</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="1">
         <v>102</v>
       </c>
-      <c r="D8" s="22">
-        <v>0</v>
-      </c>
-      <c r="E8" s="11">
+      <c r="D8" s="18">
+        <v>0</v>
+      </c>
+      <c r="E8" s="7">
         <v>7.3756635189056396</v>
       </c>
-      <c r="F8" s="10">
+      <c r="F8" s="1">
         <v>102</v>
       </c>
-      <c r="G8" s="10">
+      <c r="G8" s="1">
         <v>102</v>
       </c>
-      <c r="H8" s="22">
-        <v>0</v>
-      </c>
-      <c r="I8" s="11">
+      <c r="H8" s="18">
+        <v>0</v>
+      </c>
+      <c r="I8" s="7">
         <v>10.46786642074585</v>
       </c>
-      <c r="J8" s="10">
+      <c r="J8" s="1">
         <v>5.5</v>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="33" t="s">
+      <c r="A9" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="10">
+      <c r="B9" s="1">
         <v>86</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="1">
         <v>86</v>
       </c>
-      <c r="D9" s="22">
-        <v>0</v>
-      </c>
-      <c r="E9" s="11">
+      <c r="D9" s="18">
+        <v>0</v>
+      </c>
+      <c r="E9" s="7">
         <v>5.1456596851348877</v>
       </c>
-      <c r="F9" s="10">
+      <c r="F9" s="1">
         <v>86</v>
       </c>
-      <c r="G9" s="10">
+      <c r="G9" s="1">
         <v>86</v>
       </c>
-      <c r="H9" s="22">
-        <v>0</v>
-      </c>
-      <c r="I9" s="11">
+      <c r="H9" s="18">
+        <v>0</v>
+      </c>
+      <c r="I9" s="7">
         <v>3.3640575408935551</v>
       </c>
-      <c r="J9" s="10">
+      <c r="J9" s="1">
         <v>5.75</v>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="33" t="s">
+      <c r="A10" s="29" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="1">
         <v>81</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="1">
         <v>81</v>
       </c>
-      <c r="D10" s="22">
-        <v>0</v>
-      </c>
-      <c r="E10" s="11">
+      <c r="D10" s="18">
+        <v>0</v>
+      </c>
+      <c r="E10" s="7">
         <v>13.054975509643549</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="1">
         <v>81</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="1">
         <v>81</v>
       </c>
-      <c r="H10" s="22">
-        <v>0</v>
-      </c>
-      <c r="I10" s="11">
+      <c r="H10" s="18">
+        <v>0</v>
+      </c>
+      <c r="I10" s="7">
         <v>19.763167142868038</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="1">
         <v>6</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="34" t="s">
+      <c r="A11" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="9">
         <v>81</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="9">
         <v>81</v>
       </c>
-      <c r="D11" s="24">
-        <v>0</v>
-      </c>
-      <c r="E11" s="14">
+      <c r="D11" s="20">
+        <v>0</v>
+      </c>
+      <c r="E11" s="10">
         <v>43.315606594085693</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="9">
         <v>81</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="9">
         <v>81</v>
       </c>
-      <c r="H11" s="24">
-        <v>0</v>
-      </c>
-      <c r="I11" s="14">
+      <c r="H11" s="20">
+        <v>0</v>
+      </c>
+      <c r="I11" s="10">
         <v>49.489824295043952</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="9">
         <v>6.25</v>
       </c>
-      <c r="K11" s="15">
+      <c r="K11" s="11">
         <v>0.5</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="29" t="s">
+      <c r="A12" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="30">
-        <f>AVERAGE(B4:B11)</f>
+      <c r="B12" s="26">
+        <f t="shared" ref="B12:I12" si="0">AVERAGE(B4:B11)</f>
         <v>74.375</v>
       </c>
-      <c r="C12" s="30">
-        <f>AVERAGE(C4:C11)</f>
+      <c r="C12" s="26">
+        <f t="shared" si="0"/>
         <v>74.375</v>
       </c>
-      <c r="D12" s="31">
-        <f>AVERAGE(D4:D11)</f>
-        <v>0</v>
-      </c>
-      <c r="E12" s="30">
-        <f>AVERAGE(E4:E11)</f>
+      <c r="D12" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E12" s="26">
+        <f t="shared" si="0"/>
         <v>12.816856950521469</v>
       </c>
-      <c r="F12" s="30">
-        <f>AVERAGE(F4:F11)</f>
+      <c r="F12" s="26">
+        <f t="shared" si="0"/>
         <v>74.375</v>
       </c>
-      <c r="G12" s="30">
-        <f>AVERAGE(G4:G11)</f>
+      <c r="G12" s="26">
+        <f t="shared" si="0"/>
         <v>74.375</v>
       </c>
-      <c r="H12" s="31">
-        <f>AVERAGE(H4:H11)</f>
-        <v>0</v>
-      </c>
-      <c r="I12" s="30">
-        <f>AVERAGE(I4:I11)</f>
+      <c r="H12" s="27">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I12" s="26">
+        <f t="shared" si="0"/>
         <v>15.822187811136246</v>
       </c>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
+      <c r="J12" s="45"/>
+      <c r="K12" s="46"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:I1"/>
+  <mergeCells count="14">
+    <mergeCell ref="J12:K12"/>
     <mergeCell ref="J1:J3"/>
     <mergeCell ref="K1:K3"/>
     <mergeCell ref="B2:B3"/>
@@ -1919,6 +1992,12 @@
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:I1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>